<commit_message>
Ders içe aktarma işlemlerinde mevcudu başlığı Kontenjan/Mevcut olarak değiştirildi
</commit_message>
<xml_diff>
--- a/Public/assets/downloads/Ders Listesi.xlsx
+++ b/Public/assets/downloads/Ders Listesi.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,6 +23,49 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
+  <authors>
+    <author>Bilinmeyen Yazar</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Dersin grubu yoksa 0 yazılmalıdır.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>23</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>-228</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>17</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="90">
   <si>
@@ -50,7 +93,7 @@
     <t xml:space="preserve">Saati</t>
   </si>
   <si>
-    <t xml:space="preserve">Mevcudu</t>
+    <t xml:space="preserve">Kontenjan/Mevcut</t>
   </si>
   <si>
     <t xml:space="preserve">Hocası</t>
@@ -387,7 +430,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -417,10 +460,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -569,6 +608,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="48.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="19.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="34.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20.21"/>
   </cols>
@@ -3978,7 +4018,8 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Sayfa &amp;P</oddFooter>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -4057,7 +4098,7 @@
       <c r="E3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="6" t="s">
         <v>27</v>
       </c>
       <c r="G3" s="6"/>

</xml_diff>